<commit_message>
Sync planning SharePoint : S19
</commit_message>
<xml_diff>
--- a/Plannings 2026 S19.xlsx
+++ b/Plannings 2026 S19.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{84830FEF-CD99-488C-9111-90B341AA8F24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA600701-563D-419E-AFCD-310519774913}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{84830FEF-CD99-488C-9111-90B341AA8F24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E9CC753-6547-4148-989A-AAA1232D25F0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2759,50 +2759,6 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="50" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000032000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -6002,6 +5958,50 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1828800" y="6858000"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>124</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>124</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="125" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FEE2E840-DF84-4CBC-B6F4-0BF38063220A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3048000" y="12001500"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6380,7 +6380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H128"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6959,9 +6959,7 @@
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
-      <c r="F39" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="F39" s="4"/>
       <c r="G39" s="4" t="s">
         <v>12</v>
       </c>
@@ -6975,9 +6973,7 @@
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
-      <c r="F40" s="3" t="s">
-        <v>64</v>
-      </c>
+      <c r="F40" s="3"/>
       <c r="G40" s="3" t="s">
         <v>13</v>
       </c>
@@ -8100,6 +8096,9 @@
         <v>12</v>
       </c>
       <c r="E125" s="3"/>
+      <c r="F125" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
     </row>
@@ -8111,37 +8110,29 @@
         <v>82</v>
       </c>
       <c r="E126" s="3"/>
-      <c r="F126" s="3"/>
+      <c r="F126" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A127" s="18"/>
-      <c r="B127" s="5"/>
-      <c r="C127" s="5"/>
-      <c r="D127" s="5"/>
-      <c r="E127" s="5"/>
-      <c r="F127" s="5"/>
-      <c r="G127" s="5"/>
-      <c r="H127" s="5"/>
-    </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B128" s="19"/>
-      <c r="C128" s="19"/>
-      <c r="D128" s="19"/>
-      <c r="E128" s="19"/>
-      <c r="F128" s="19"/>
-      <c r="G128" s="19"/>
-      <c r="H128" s="19"/>
+      <c r="B127" s="19"/>
+      <c r="C127" s="19"/>
+      <c r="D127" s="19"/>
+      <c r="E127" s="19"/>
+      <c r="F127" s="19"/>
+      <c r="G127" s="19"/>
+      <c r="H127" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B128:H128"/>
+    <mergeCell ref="B127:H127"/>
     <mergeCell ref="A107:A109"/>
     <mergeCell ref="A110:A114"/>
     <mergeCell ref="A115:A117"/>
     <mergeCell ref="A118:A124"/>
-    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="A125:A126"/>
     <mergeCell ref="A78:A82"/>
     <mergeCell ref="A83:A91"/>
     <mergeCell ref="A92:A95"/>
@@ -8935,13 +8926,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1F483C7-9028-4F57-B9B2-0A1FA1490184}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E892E56B-4DB9-4737-87C8-68381ACFF402}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C3B6EAD-CC4B-4575-B2E1-0204E1EA0456}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CB6A53DC-7929-40D2-9B98-EC353EFBC1E5}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D1BC428-03DB-41A1-B8B5-2FAC2A2749FD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8A8CB62-EC1E-4BD8-BBB5-8A7D85090CA9}"/>
 </file>
</xml_diff>